<commit_message>
October Dispatch (Issue #5): Field Notes revisions, Clinton trip report, food-storage title; site-wide new-tab external links and Newsletter nav label
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -513,7 +513,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carriers: 68 rows, 12 columns.</t>
+          <t>Carriers: 69 rows, 12 columns.</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Of the 68 carriers here, 33 have had their bicycle policy checked against the operator's own material, 7 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
+          <t>Of the 69 carriers here, 33 have had their bicycle policy checked against the operator's own material, 8 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3160,19 +3160,19 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>VIA Rail</t>
+          <t>Tunnel49</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>intercity-train</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Checked baggage (staffed stations only, including Vancouver BC and Jasper AB); $25 per direction; E-bikes OK (battery disconnected at check-in)</t>
+          <t>Rides in the hold (boxed, bagged, or wrapped); Bike fee ($50 + GST per bike bag on the Calgary shuttle; Cranbrook might be extra)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3191,41 +3191,36 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>listing-description</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/4cb8d28c4b/</t>
+          <t>https://bccycletourism.ca/wwc/stop/7f19847d08/</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.viarail.ca</t>
+          <t>https://t49.ca</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Victoria Clipper</t>
+          <t>VIA Rail</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ferry</t>
+          <t>intercity-train</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3234,17 +3229,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Reserve ahead by phone (space very limited, first booked first served); $30 USD each way (about $41 CAD); Rides on the open deck (bags and accessories off; waiver at check-in)</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Rides on the open deck (bags and accessories off; waiver at check-in)</t>
+          <t>Checked baggage (staffed stations only, including Vancouver BC and Jasper AB); $25 per direction; E-bikes OK (battery disconnected at check-in)</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3254,52 +3244,82 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/f217a1bbde/</t>
+          <t>https://bccycletourism.ca/wwc/stop/4cb8d28c4b/</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.clippervacations.com</t>
+          <t>https://www.viarail.ca</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Victoria Harbour Ferry</t>
+          <t>Victoria Clipper</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Reserve ahead by phone (space very limited, first booked first served); $30 USD each way (about $41 CAD); Rides on the open deck (bags and accessories off; waiver at check-in)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Rides on the open deck (bags and accessories off; waiver at check-in)</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/f217a1bbde/</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://www.clippervacations.com</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>West Coast Launch</t>
+          <t>Victoria Harbour Ferry</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3308,10 +3328,10 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -3321,189 +3341,159 @@
       <c r="I61" t="inlineStr">
         <is>
           <t>not-on-file</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/22a5ae41f3/</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>https://www.westcoastlaunch.com/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>West Coast Trail Express</t>
+          <t>West Coast Launch</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D62" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/5117c40285/</t>
+          <t>https://bccycletourism.ca/wwc/stop/22a5ae41f3/</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://trailbus.com/</t>
+          <t>https://www.westcoastlaunch.com/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>West Coast Transit System (Tofino/Ucluelet)</t>
+          <t>West Coast Trail Express</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>local-bus</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Rack on the bus, free (2 bikes · first come, first served); E-bikes OK</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>none</t>
+          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
+          <t>https://bccycletourism.ca/wwc/stop/5117c40285/</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.bctransit.com</t>
+          <t>https://trailbus.com/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>WestJet</t>
+          <t>West Coast Transit System (Tofino/Ucluelet)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>local-bus</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Box or sturdy bag required; Bike fee; No e-bikes</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Box or sturdy bag required; No e-bikes</t>
+          <t>Rack on the bus, free (2 bikes · first come, first served); E-bikes OK</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>none</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>listing-description</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/b5f48a88ff/</t>
+          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.westjet.com</t>
+          <t>https://www.bctransit.com</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Whistler Shuttle</t>
+          <t>WestJet</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3512,12 +3502,17 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Book ahead (bikes carried with advance notice); Bike fee</t>
+          <t>Box or sturdy bag required; Bike fee; No e-bikes</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Box or sturdy bag required; No e-bikes</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>preparation</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3532,100 +3527,100 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/c7e12671ea/</t>
+          <t>https://bccycletourism.ca/wwc/stop/b5f48a88ff/</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.whistlershuttle.com</t>
+          <t>https://www.westjet.com</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Wilderness Seaplanes</t>
+          <t>Whistler Shuttle</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Book ahead (bikes carried with advance notice); Bike fee</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/c7e12671ea/</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://www.whistlershuttle.com</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Wilson's Transportation (BC Connector)</t>
+          <t>Wilderness Seaplanes</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Rides in the hold (bagged or boxed); $42 per bike (50 lb max); Reserve bike spot (recommended)</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/ca9171f28f/</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>https://wilsonstransportation.com/</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>YVR Skylynx</t>
+          <t>Wilson's Transportation (BC Connector)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3646,7 +3641,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Rides in the hold (bagged, wrapped, or boxed); First bike free; Reserve ahead (Squamish is reservation-only)</t>
+          <t>Rides in the hold (bagged or boxed); $42 per bike (50 lb max); Reserve bike spot (recommended)</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3666,38 +3661,91 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/49b1ded455/</t>
+          <t>https://bccycletourism.ca/wwc/stop/ca9171f28f/</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.yvrskylynx.com</t>
+          <t>https://wilsonstransportation.com/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>YVR Skylynx</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Rides in the hold (bagged, wrapped, or boxed); First bike free; Reserve ahead (Squamish is reservation-only)</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>preparation</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/49b1ded455/</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>https://www.yvrskylynx.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
           <t>Zeballos Expeditions (Zeballos Water Taxi)</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>water-taxi</t>
         </is>
       </c>
-      <c r="C69" t="n">
-        <v>1</v>
-      </c>
-      <c r="D69" t="n">
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
         <v>0</v>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I70" t="inlineStr">
         <is>
           <t>not-on-file</t>
         </is>

</xml_diff>

<commit_message>
October Dispatch: issue date Oct 8
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -3169,10 +3169,10 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Transit map, number refresh, campground   seasons, To and Fro fix
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -462,7 +462,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Published 2026-10-08 by BC Cycle Tourism Society.</t>
+          <t>Published 2026-10-18 by BC Cycle Tourism Society.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-10-08. https://bccycletourism.ca/research/</t>
+          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-10-18. https://bccycletourism.ca/research/</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carriers: 69 rows, 12 columns.</t>
+          <t>Carriers: 72 rows, 12 columns.</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Of the 69 carriers here, 33 have had their bicycle policy checked against the operator's own material, 8 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
+          <t>Of the 72 carriers here, 36 have had their bicycle policy checked against the operator's own material, 8 are read from the operator's published description and not separately checked, and 28 have no bicycle policy on file at all. That last group is a finding, not an oversight: for much of British Columbia, nobody publishes this anywhere.</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -714,10 +714,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alaska Airlines</t>
+          <t>Air North</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -772,10 +772,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -784,12 +784,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Rides in the hold (boxed, bagged, or wrapped); Bike fee; No e-bikes</t>
+          <t>Hard case or bike box (a box needs a signed release; 32 kg max); $50 plus tax; Add your bike to the booking ahead (space available); E-bikes only with a small battery (removable, 160 Wh max, carried in the cabin)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No e-bikes</t>
+          <t>E-bikes only with a small battery (removable, 160 Wh max, carried in the cabin)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -799,29 +799,34 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/05ad4bc89f/</t>
+          <t>https://bccycletourism.ca/wwc/stop/d08b1306bd/</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.alaskaair.com/</t>
+          <t>https://flyairnorth.com/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Amtrak Cascades</t>
+          <t>Alaska Airlines</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>intercity-train</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -837,44 +842,44 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Roll on the bike car; Reserve bike spot; Bike fee</t>
+          <t>Rides in the hold (boxed, bagged, or wrapped); Bike fee; No e-bikes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No e-bikes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>preparation</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>listing-description</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/e73d52aff2/</t>
+          <t>https://bccycletourism.ca/wwc/stop/05ad4bc89f/</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://amtrakcascades.com/</t>
+          <t>https://www.alaskaair.com/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BC Bus North (Tahltan NST Busing Ltd.)</t>
+          <t>Alaska Marine Highway</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -890,12 +895,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Luggage bay on the Prince Rupert route; Other routes: bagged or boxed (checked as luggage)</t>
+          <t>Roll on, ready to ride (no boxed or taken-apart bikes); Bike fare (not published; call 1-800-642-0066); E-bikes OK (push it on and off the ramp)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>preparation</t>
+          <t>fee</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -905,50 +910,50 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/59ccc68831/</t>
+          <t>https://bccycletourism.ca/wwc/stop/bc8da050ed/</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.tnst.ca/bc-bus-north/passenger-information</t>
+          <t>https://dot.alaska.gov/amhs/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BC Ferries</t>
+          <t>Amtrak Cascades</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ferry</t>
+          <t>intercity-train</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>yes, with conditions</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Roll on, free (no reservation needed); E-bikes OK (no charging on board)</t>
+          <t>Roll on the bike car; Reserve bike spot; Bike fee</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -963,98 +968,98 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/b06e4282f9/</t>
+          <t>https://bccycletourism.ca/wwc/stop/e73d52aff2/</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.bcferries.com</t>
+          <t>https://amtrakcascades.com/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BC Inland Ferries</t>
+          <t>BC Bus North (Tahltan NST Busing Ltd.)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>inland-ferry</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>yes, with conditions</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Roll on; E-bikes OK</t>
+          <t>Luggage bay on the Prince Rupert route; Other routes: bagged or boxed (checked as luggage)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/96591f20f2/</t>
+          <t>https://bccycletourism.ca/wwc/stop/59ccc68831/</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www2.gov.bc.ca/gov/content/transportation/passenger-travel/water-travel/inland-ferries/kootenay-lake-ferry</t>
+          <t>https://www.tnst.ca/bc-bus-north/passenger-information</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BC Transit</t>
+          <t>BC Ferries</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>bus; local-bus</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>94</v>
+        <v>25</v>
       </c>
       <c r="D9" t="n">
-        <v>94</v>
+        <v>25</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Front rack, no fee (2 bikes, first come; space not guaranteed); E-bikes under 25 kg only (lithium battery off the bike and carried on board)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>E-bikes under 25 kg only (lithium battery off the bike and carried on board)</t>
+          <t>Roll on, free (no reservation needed); E-bikes OK (no charging on board)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>none</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1064,133 +1069,158 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
+          <t>https://bccycletourism.ca/wwc/stop/b06e4282f9/</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.bctransit.com</t>
+          <t>https://www.bcferries.com</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BLAST (English Bay Launch)</t>
+          <t>BC Inland Ferries</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>inland-ferry</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Roll on; E-bikes OK</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>listing-description</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/96591f20f2/</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www2.gov.bc.ca/gov/content/transportation/passenger-travel/water-travel/inland-ferries/kootenay-lake-ferry</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Blind Channel Water Taxi</t>
+          <t>BC Transit</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>bus; local-bus</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Front rack, no fee (2 bikes, first come; space not guaranteed); E-bikes under 25 kg only (lithium battery off the bike and carried on board)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>E-bikes under 25 kg only (lithium battery off the bike and carried on board)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.bctransit.com</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>BLAST (English Bay Launch)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>rental-car</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>One-way between BC Budget branches (bookable online); Bike rides inside (SUV or minivan, seats folded, wheels off); Confirm one-way and vehicle when booking</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/a60b8f9cd0/</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>https://www.avis.ca</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cape Scott Water Taxi (North Coast Trail Shuttle)</t>
+          <t>Blind Channel Water Taxi</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1199,7 +1229,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -1214,49 +1244,64 @@
           <t>not-on-file</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/bf5c8df747/</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>https://www.capescottwatertaxi.ca/</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Central Mountain Air</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>rental-car</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>One-way between BC Budget branches (bookable online); Bike rides inside (SUV or minivan, seats folded, wheels off); Confirm one-way and vehicle when booking</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/a60b8f9cd0/</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.avis.ca</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cormorant Marine Water Taxi</t>
+          <t>Cape Scott Water Taxi (North Coast Trail Shuttle)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1265,7 +1310,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -1280,23 +1325,33 @@
           <t>not-on-file</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/bf5c8df747/</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.capescottwatertaxi.ca/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Discovery Launch Water Taxi</t>
+          <t>Central Mountain Air</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1306,23 +1361,13 @@
       <c r="I16" t="inlineStr">
         <is>
           <t>not-on-file</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/cc33103e57/</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>https://discoverylaunch.com/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Discovery West Adventures</t>
+          <t>Cormorant Marine Water Taxi</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1331,7 +1376,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -1350,113 +1395,73 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ebus</t>
+          <t>Discovery Launch Water Taxi</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Rides in the hold (bagged or cloth-wrapped (no plastic), or boxed); $30 per bike</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/af77874ba6/</t>
+          <t>https://bccycletourism.ca/wwc/stop/cc33103e57/</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.myebus.ca</t>
+          <t>https://discoverylaunch.com/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Electric Alpine Biking</t>
+          <t>Discovery West Adventures</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>local-bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Bring your own bike ($19 one-way pass, no extra bike fee); Book ahead (seats may be limited)</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/8436067ac9/</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>https://electricalpine.com</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Epic Rides</t>
+          <t>Ebus</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1465,10 +1470,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1477,7 +1482,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bikes ride free (outside rack, or boxed under the bus); Box to avoid scratches (outside-rack bikes ride at your own risk)</t>
+          <t>Rides in the hold (bagged or cloth-wrapped (no plastic), or boxed); $30 per bike</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1497,31 +1502,31 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/ff02318a56/</t>
+          <t>https://bccycletourism.ca/wwc/stop/af77874ba6/</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://epicrides.ca</t>
+          <t>https://www.myebus.ca</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Flair Airlines</t>
+          <t>Electric Alpine Biking</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>local-bus</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1530,39 +1535,39 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Rides in the hold (boxed, bagged, or wrapped); Bike fee; Reserve bike spot; No e-bikes</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>No e-bikes</t>
+          <t>Bring your own bike ($19 one-way pass, no extra bike fee); Book ahead (seats may be limited)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/8756f55c9e/</t>
+          <t>https://bccycletourism.ca/wwc/stop/8436067ac9/</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.flyflair.com/</t>
+          <t>https://electricalpine.com</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FlixBus (operated by MTRWestern)</t>
+          <t>Epic Rides</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1583,17 +1588,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Rack on the bus (space not guaranteed); About $19–37; Book bike as add-on; No e-bikes, tandems or trailers</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>No e-bikes, tandems or trailers</t>
+          <t>Bikes ride free (outside rack, or boxed under the bus); Box to avoid scratches (outside-rack bikes ride at your own risk)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1608,45 +1608,50 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/af3d5bbd19/</t>
+          <t>https://bccycletourism.ca/wwc/stop/ff02318a56/</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.flixbus.ca</t>
+          <t>https://epicrides.ca</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>George Massey Tunnel Bike Shuttle</t>
+          <t>Flair Airlines</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>local-bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>yes, with conditions</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>E-bikes OK</t>
+          <t>Rides in the hold (boxed, bagged, or wrapped); Bike fee; Reserve bike spot; No e-bikes</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No e-bikes</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1656,31 +1661,31 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/b65c89ee1c/</t>
+          <t>https://bccycletourism.ca/wwc/stop/8756f55c9e/</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.gov.bc.ca/george-massey-shuttle</t>
+          <t>https://www.flyflair.com/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Harbour Air</t>
+          <t>FlixBus (operated by MTRWestern)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1689,12 +1694,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Front wheel must come off; $20 handling fee (bike weight counts toward your baggage allowance); Not on the Twin Otter (other floatplanes are fine; confirm when booking)</t>
+          <t>Rack on the bus (space not guaranteed); About $19–37; Book bike as add-on; No e-bikes, tandems or trailers</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Not on the Twin Otter (other floatplanes are fine; confirm when booking)</t>
+          <t>No e-bikes, tandems or trailers</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1714,59 +1719,79 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/f6d9ce9479/</t>
+          <t>https://bccycletourism.ca/wwc/stop/af3d5bbd19/</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.harbourair.com</t>
+          <t>https://www.flixbus.ca</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Helijet</t>
+          <t>George Massey Tunnel Bike Shuttle</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>local-bus</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>E-bikes OK</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>listing-description</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/b65c89ee1c/</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.gov.bc.ca/george-massey-shuttle</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Hullo</t>
+          <t>Harbour Air</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ferry</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1775,12 +1800,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Book online ahead (6 bike spots per sailing, 1 per guest); $19.99 one way ($25 in person); No e-bikes (no trailers, 80 in / 50 lb max)</t>
+          <t>Front wheel must come off; $20 handling fee (bike weight counts toward your baggage allowance); Not on the Twin Otter (other floatplanes are fine; confirm when booking)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No e-bikes (no trailers, 80 in / 50 lb max)</t>
+          <t>Not on the Twin Otter (other floatplanes are fine; confirm when booking)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1800,72 +1825,52 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/e8324765f2/</t>
+          <t>https://bccycletourism.ca/wwc/stop/f6d9ce9479/</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.hullo.com</t>
+          <t>https://www.harbourair.com</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Island Link</t>
+          <t>Helijet</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/42fea27c49/</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>https://islandlinkbus.com</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Lasqueti Island Ferry (Western Pacific Marine)</t>
+          <t>Hullo</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1881,72 +1886,92 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Bike fee</t>
+          <t>Book online ahead (6 bike spots per sailing, 1 per guest); $19.99 one way ($25 in person); No e-bikes (no trailers, 80 in / 50 lb max)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No e-bikes (no trailers, 80 in / 50 lb max)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>fee</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/84661e6aae/</t>
+          <t>https://bccycletourism.ca/wwc/stop/e8324765f2/</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://westernpacificmarine.com/routes/lasqueti-island/</t>
+          <t>https://www.hullo.com</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lund Water Taxi</t>
+          <t>Island Link</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/f6e2b04bf0/</t>
+          <t>https://bccycletourism.ca/wwc/stop/42fea27c49/</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.lundwatertaxi.com/</t>
+          <t>https://islandlinkbus.com</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MV Uchuck III (Nootka Sound Service Ltd / Get West)</t>
+          <t>Lasqueti Island Ferry (Western Pacific Marine)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1955,36 +1980,46 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Bike fee</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>fee</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>listing-description</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/7640e33a07/</t>
+          <t>https://bccycletourism.ca/wwc/stop/84661e6aae/</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://getwest.ca/cruises/schedule/</t>
+          <t>https://westernpacificmarine.com/routes/lasqueti-island/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Metlakatla Ferry Service</t>
+          <t>Lund Water Taxi</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1993,7 +2028,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
         <v>1</v>
@@ -2010,24 +2045,24 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/fb6715dfdd/</t>
+          <t>https://bccycletourism.ca/wwc/stop/f6e2b04bf0/</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.metlakatla.ca/metlakatla-ferry-service/ferry-schedule</t>
+          <t>https://www.lundwatertaxi.com/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mountain Man Mike's</t>
+          <t>MV Uchuck III (Nootka Sound Service Ltd / Get West)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -2038,109 +2073,79 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Bikes accepted; Call for a quote (fee and packaging arranged with the booking agent)</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/9694f0f95d/</t>
+          <t>https://bccycletourism.ca/wwc/stop/7640e33a07/</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://mountainmanmikes.ca/</t>
+          <t>https://getwest.ca/cruises/schedule/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>National Car &amp; Truck Rental (Vancouver Island)</t>
+          <t>Metlakatla Ferry Service</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>rental-car</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>One-way between Island branches (no drop charge); Bike rides inside (SUV or minivan, seats folded, wheels off); Confirm one-way and vehicle when booking</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/77b9f3315a/</t>
+          <t>https://bccycletourism.ca/wwc/stop/fb6715dfdd/</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.drivenational.ca</t>
+          <t>https://www.metlakatla.ca/metlakatla-ferry-service/ferry-schedule</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Newcastle Island Ferry Service LP</t>
+          <t>Mountain Man Mike's</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ferry</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2149,79 +2154,104 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Roll on; Bike fee ($5 (kids) / $7 (adult), return); No e-bikes</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>No e-bikes</t>
+          <t>Bikes accepted; Call for a quote (fee and packaging arranged with the booking agent)</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/d5f417c1c2/</t>
+          <t>https://bccycletourism.ca/wwc/stop/9694f0f95d/</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://newcastleisland.ca/schedule</t>
+          <t>https://mountainmanmikes.ca/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Nootka Water Taxi</t>
+          <t>National Car &amp; Truck Rental (Vancouver Island)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>rental-car</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>One-way between Island branches (no drop charge); Bike rides inside (SUV or minivan, seats folded, wheels off); Confirm one-way and vehicle when booking</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/77b9f3315a/</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.drivenational.ca</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Pacific Coastal Airlines</t>
+          <t>Newcastle Island Ferry Service LP</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2230,7 +2260,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Rides in the hold (small aircraft, limited space); About $105 per direction; No e-bikes</t>
+          <t>Roll on; Bike fee ($5 (kids) / $7 (adult), return); No e-bikes</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2245,137 +2275,122 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>listing-description</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/37d712c454/</t>
+          <t>https://bccycletourism.ca/wwc/stop/d5f417c1c2/</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.pacificcoastal.com</t>
+          <t>https://newcastleisland.ca/schedule</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Poparide</t>
+          <t>Nootka Water Taxi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>carpool</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Only some rides take bikes (look for the bicycle icon on the listing); Schedule is variable (check Poparide for driver-listed dates and times)</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Only some rides take bikes (look for the bicycle icon on the listing); Schedule is variable (check Poparide for driver-listed dates and times)</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>restriction</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/251538fa02/</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>https://www.poparide.com/</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Qaya Way West Transportation</t>
+          <t>Pacific Coastal Airlines</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Rides in the hold (small aircraft, limited space); About $105 per direction; No e-bikes</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>No e-bikes</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/a71df6016c/</t>
+          <t>https://bccycletourism.ca/wwc/stop/37d712c454/</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://waywest.ca/</t>
+          <t>https://www.pacificcoastal.com</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Quick Shuttle (Quick Coach Lines / TRAXX)</t>
+          <t>Poparide</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>carpool</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2384,12 +2399,17 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Bikes accepted (book as an add-on); $42 USD each (about $57 CAD)</t>
+          <t>Only some rides take bikes (look for the bicycle icon on the listing); Schedule is variable (check Poparide for driver-listed dates and times)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Only some rides take bikes (look for the bicycle icon on the listing); Schedule is variable (check Poparide for driver-listed dates and times)</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>fee</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2404,24 +2424,24 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/cfa3ab3785/</t>
+          <t>https://bccycletourism.ca/wwc/stop/251538fa02/</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://quickcoach.com/en</t>
+          <t>https://www.poparide.com/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rider Express</t>
+          <t>Qaya Way West Transportation</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2432,112 +2452,147 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Rides in the hold (bagged, wrapped, or boxed); $50 per bike (non-refundable)</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/85f8ab1d65/</t>
+          <t>https://bccycletourism.ca/wwc/stop/a71df6016c/</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.riderexpress.ca</t>
+          <t>https://waywest.ca/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Saltspring Air</t>
+          <t>Quick Shuttle (Quick Coach Lines / TRAXX)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Bikes accepted (book as an add-on); $42 USD each (about $57 CAD)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>fee</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/cfa3ab3785/</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://quickcoach.com/en</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Savary Island Ferry (Finn Bay Marine / Access Point Marine)</t>
+          <t>Rider Express</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Rides in the hold (bagged, wrapped, or boxed); $50 per bike (non-refundable)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/85f8ab1d65/</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.riderexpress.ca</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SeaCoastal Water Taxi (Kitasoo Xai'xais)</t>
+          <t>Saltspring Air</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2547,32 +2602,22 @@
       <c r="I43" t="inlineStr">
         <is>
           <t>not-on-file</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/a3918eb8be/</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>https://klemtutaxi.com/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Seair Seaplanes</t>
+          <t>Savary Island Ferry (Finn Bay Marine / Access Point Marine)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -2591,7 +2636,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Shorebird Expeditions</t>
+          <t>SeaCoastal Water Taxi (Kitasoo Xai'xais)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2600,10 +2645,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2613,119 +2658,79 @@
       <c r="I45" t="inlineStr">
         <is>
           <t>not-on-file</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/a3918eb8be/</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://klemtutaxi.com/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Silver City Stagelines</t>
+          <t>Seair Seaplanes</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/e9065ae25e/</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>https://fritztravels.com/</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Squamish Connector</t>
+          <t>Shorebird Expeditions</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C47" t="n">
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Book ahead; Max 2 bikes per trip; Some buses have an outside rack (otherwise carried in the luggage hold); $15 each way; No e-bikes</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>No e-bikes</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>restriction</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/a3a6b94ea1/</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>https://www.squamishconnector.com</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sunshine Coast Connector</t>
+          <t>Silver City Stagelines</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2741,17 +2746,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Reserve bike spot (rack space is limited); $20 bike · $40 e-bike; No box needed (rack on the bus)</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2761,24 +2761,24 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/653ad042f7/</t>
+          <t>https://bccycletourism.ca/wwc/stop/e9065ae25e/</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.sunshinecoastconnector.ca/</t>
+          <t>https://fritztravels.com/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Sunshine Coast Shuttle</t>
+          <t>Squamish Connector</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2790,66 +2790,111 @@
         <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Book ahead; Max 2 bikes per trip; Some buses have an outside rack (otherwise carried in the luggage hold); $15 each way; No e-bikes</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No e-bikes</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/a5117520f3/</t>
+          <t>https://bccycletourism.ca/wwc/stop/a3a6b94ea1/</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://sunshinecoastshuttle.ca/</t>
+          <t>https://www.squamishconnector.com</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Sutil Charters</t>
+          <t>Sunshine Coast Connector</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Reserve bike spot (rack space is limited); $20 bike · $40 e-bike; No box needed (rack on the bus)</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/653ad042f7/</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://www.sunshinecoastconnector.ca/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Terracentric Coastal Adventures</t>
+          <t>Sunshine Coast Shuttle</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2868,11 +2913,21 @@
           <t>not-on-file</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/a5117520f3/</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>https://sunshinecoastshuttle.ca/</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Tofino Water Taxi</t>
+          <t>Sutil Charters</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2900,125 +2955,75 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TransLink</t>
+          <t>Terracentric Coastal Adventures</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>local-bus; skytrain</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Rack on the bus, free; 2 bikes (first come, first served); E-bikes OK</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/6ee82dcb4e/</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>https://www.translink.ca/rider-guide/bike-and-ride-on-transit/bikes-on-transit</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TransLink (Coast Mountain Bus Co.)</t>
+          <t>Tofino Water Taxi</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>local-bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C54" t="n">
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Rack on the bus, free; 2 bikes (first come, first served); E-bikes OK</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/6ee82dcb4e/</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>https://www.translink.ca/rider-guide/bike-and-ride-on-transit/bikes-on-transit</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TransLink (SeaBus)</t>
+          <t>TransLink</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ferry</t>
+          <t>local-bus; skytrain</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D55" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -3027,17 +3032,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Roll on, free (bikes ride inside the cabin); 6 bikes per sailing at rush hour (weekdays 7–9:30 am and 3–6:30 pm; no limit other times); E-bikes OK (no charging on board); No trailers (185 cm max bike length)</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>No trailers (185 cm max bike length)</t>
+          <t>Rack on the bus, free; 2 bikes (first come, first served); E-bikes OK</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3047,29 +3047,29 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/60eab20168/</t>
+          <t>https://bccycletourism.ca/wwc/stop/6ee82dcb4e/</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.translink.ca/rider-guide/bikes-on-transit/seabus</t>
+          <t>https://www.translink.ca/rider-guide/bike-and-ride-on-transit/bikes-on-transit</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TransLink (West Coast Express)</t>
+          <t>TransLink (Coast Mountain Bus Co.)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>local-train</t>
+          <t>local-bus</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3085,17 +3085,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Roll on, free (2 bikes per car); Weekdays only (peak direction only)</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Weekdays only (peak direction only)</t>
+          <t>Rack on the bus, free; 2 bikes (first come, first served); E-bikes OK</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>restriction</t>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3122,12 +3117,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Tsimshian Storm (Kitkatla/Hartley Bay/Metlakatla)</t>
+          <t>TransLink (SeaBus)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3138,41 +3133,61 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Roll on, free (bikes ride inside the cabin); 6 bikes per sailing at rush hour (weekdays 7–9:30 am and 3–6:30 pm; no limit other times); E-bikes OK (no charging on board); No trailers (185 cm max bike length)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No trailers (185 cm max bike length)</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/408314e58c/</t>
+          <t>https://bccycletourism.ca/wwc/stop/60eab20168/</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://gitxaalanation.com/ferries/</t>
+          <t>https://www.translink.ca/rider-guide/bikes-on-transit/seabus</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Tunnel49</t>
+          <t>TransLink (West Coast Express)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>local-train</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -3181,46 +3196,56 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Rides in the hold (boxed, bagged, or wrapped); Bike fee ($50 + GST per bike bag on the Calgary shuttle; Cranbrook might be extra)</t>
+          <t>Roll on, free (2 bikes per car); Weekdays only (peak direction only)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Weekdays only (peak direction only)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>preparation</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>listing-description</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/7f19847d08/</t>
+          <t>https://bccycletourism.ca/wwc/stop/6ee82dcb4e/</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://t49.ca</t>
+          <t>https://www.translink.ca/rider-guide/bike-and-ride-on-transit/bikes-on-transit</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>VIA Rail</t>
+          <t>Tsal'alh Seton Train</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>intercity-train</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3229,7 +3254,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Checked baggage (staffed stations only, including Vancouver BC and Jasper AB); $25 per direction; E-bikes OK (battery disconnected at check-in)</t>
+          <t>Bikes ride along ($2.50 each way); Check before you go (schedule changes and closures are posted on Facebook; call (250) 259-8300)</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3244,29 +3269,29 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/4cb8d28c4b/</t>
+          <t>https://bccycletourism.ca/wwc/stop/1b7111508a/</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.viarail.ca</t>
+          <t>https://www.facebook.com/Kaoham2022</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Victoria Clipper</t>
+          <t>Tsimshian Storm (Kitkatla/Hartley Bay/Metlakatla)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ferry</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -3277,136 +3302,161 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Reserve ahead by phone (space very limited, first booked first served); $30 USD each way (about $41 CAD); Rides on the open deck (bags and accessories off; waiver at check-in)</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>Rides on the open deck (bags and accessories off; waiver at check-in)</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>restriction</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/f217a1bbde/</t>
+          <t>https://bccycletourism.ca/wwc/stop/408314e58c/</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.clippervacations.com</t>
+          <t>https://gitxaalanation.com/ferries/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Victoria Harbour Ferry</t>
+          <t>Tunnel49</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>2</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Rides in the hold (boxed, bagged, or wrapped); Bike fee ($50 + GST per bike bag on the Calgary shuttle; Cranbrook might be extra)</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>listing-description</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/7f19847d08/</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>https://t49.ca</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>West Coast Launch</t>
+          <t>VIA Rail</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>intercity-train</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Checked baggage (staffed stations only, including Vancouver BC and Jasper AB); $25 per direction; E-bikes OK (battery disconnected at check-in)</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>preparation</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/22a5ae41f3/</t>
+          <t>https://bccycletourism.ca/wwc/stop/4cb8d28c4b/</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.westcoastlaunch.com/</t>
+          <t>https://www.viarail.ca</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>West Coast Trail Express</t>
+          <t>Victoria Clipper</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>ferry</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes, with conditions</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
+          <t>Reserve ahead by phone (space very limited, first booked first served); $30 USD each way (about $41 CAD); Rides on the open deck (bags and accessories off; waiver at check-in)</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Rides on the open deck (bags and accessories off; waiver at check-in)</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3416,130 +3466,90 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/5117c40285/</t>
+          <t>https://bccycletourism.ca/wwc/stop/f217a1bbde/</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://trailbus.com/</t>
+          <t>https://www.clippervacations.com</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>West Coast Transit System (Tofino/Ucluelet)</t>
+          <t>Victoria Harbour Ferry</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>local-bus</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Rack on the bus, free (2 bikes · first come, first served); E-bikes OK</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>none</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>listing-description</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>https://www.bctransit.com</t>
+          <t>not-on-file</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>WestJet</t>
+          <t>West Coast Launch</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>water-taxi</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D65" t="n">
         <v>4</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Box or sturdy bag required; Bike fee; No e-bikes</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>Box or sturdy bag required; No e-bikes</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>restriction</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>operator-checked</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
+          <t>not-on-file</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/b5f48a88ff/</t>
+          <t>https://bccycletourism.ca/wwc/stop/22a5ae41f3/</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.westjet.com</t>
+          <t>https://www.westcoastlaunch.com/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Whistler Shuttle</t>
+          <t>West Coast Trail Express</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3548,24 +3558,19 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>yes, with conditions</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Book ahead (bikes carried with advance notice); Bike fee</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>preparation</t>
+          <t>Bikes are not carried on this operator's services. We checked this one specifically.</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3575,64 +3580,84 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/c7e12671ea/</t>
+          <t>https://bccycletourism.ca/wwc/stop/5117c40285/</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.whistlershuttle.com</t>
+          <t>https://trailbus.com/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Wilderness Seaplanes</t>
+          <t>West Coast Transit System (Tofino/Ucluelet)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>air</t>
+          <t>local-bus</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Rack on the bus, free (2 bikes · first come, first served); E-bikes OK</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>not-on-file</t>
+          <t>listing-description</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/da412616ad/</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>https://www.bctransit.com</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Wilson's Transportation (BC Connector)</t>
+          <t>WestJet</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D68" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3641,12 +3666,17 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Rides in the hold (bagged or boxed); $42 per bike (50 lb max); Reserve bike spot (recommended)</t>
+          <t>Box or sturdy bag required; Bike fee; No e-bikes</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Box or sturdy bag required; No e-bikes</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>preparation</t>
+          <t>restriction</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3661,19 +3691,19 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/ca9171f28f/</t>
+          <t>https://bccycletourism.ca/wwc/stop/b5f48a88ff/</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://wilsonstransportation.com/</t>
+          <t>https://www.westjet.com</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>YVR Skylynx</t>
+          <t>Whistler Shuttle</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3694,7 +3724,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Rides in the hold (bagged, wrapped, or boxed); First bike free; Reserve ahead (Squamish is reservation-only)</t>
+          <t>Book ahead (bikes carried with advance notice); Bike fee</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3714,28 +3744,28 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>https://bccycletourism.ca/wwc/stop/49b1ded455/</t>
+          <t>https://bccycletourism.ca/wwc/stop/c7e12671ea/</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.yvrskylynx.com</t>
+          <t>https://www.whistlershuttle.com</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Zeballos Expeditions (Zeballos Water Taxi)</t>
+          <t>Wilderness Seaplanes</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>water-taxi</t>
+          <t>air</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -3746,6 +3776,140 @@
         </is>
       </c>
       <c r="I70" t="inlineStr">
+        <is>
+          <t>not-on-file</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Wilson's Transportation (BC Connector)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Rides in the hold (bagged or boxed); $42 per bike (50 lb max); Reserve bike spot (recommended)</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>preparation</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/ca9171f28f/</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>https://wilsonstransportation.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>YVR Skylynx</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>yes, with conditions</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Rides in the hold (bagged, wrapped, or boxed); First bike free; Reserve ahead (Squamish is reservation-only)</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>preparation</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>operator-checked</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>https://bccycletourism.ca/wwc/stop/49b1ded455/</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.yvrskylynx.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Zeballos Expeditions (Zeballos Water Taxi)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>water-taxi</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
         <is>
           <t>not-on-file</t>
         </is>

</xml_diff>

<commit_message>
To and Fro: weekly-only and no-rental keepers (Hope-Princeton via Kelowna), flight title drops 'scenic'; transit research numbers refreshed; Trans Canada Trail comfort map (unlinked)
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_carriers.xlsx
+++ b/research/files/bc_transit_carriers.xlsx
@@ -462,7 +462,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Published 2026-10-18 by BC Cycle Tourism Society.</t>
+          <t>Published 2026-10-20 by BC Cycle Tourism Society.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-10-18. https://bccycletourism.ca/research/</t>
+          <t>Suggested citation: BC Cycle Tourism Society (2026). British Columbia carriers and their bicycle policies [data set]. Version 2026-10-20. https://bccycletourism.ca/research/</t>
         </is>
       </c>
     </row>

</xml_diff>